<commit_message>
New sng objective etc.
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -538,7 +538,7 @@
     <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
@@ -570,7 +570,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -596,8 +596,12 @@
       <c r="L2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O2">
+        <f>K2/J2</f>
+        <v>0.95517385839966484</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -623,8 +627,12 @@
       <c r="L3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O3">
+        <f>K3/J3</f>
+        <v>0.95652916559911172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -652,7 +660,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -680,7 +688,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -707,7 +715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -734,7 +742,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -766,7 +774,7 @@
       </c>
       <c r="M11" s="6"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -779,7 +787,7 @@
       <c r="K12" s="4"/>
       <c r="M12" s="6"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>32</v>
       </c>
@@ -795,7 +803,7 @@
       <c r="K13" s="4"/>
       <c r="M13" s="6"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -825,7 +833,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -846,7 +854,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Updated scenario data based on latest from Karin (slight adjustments)
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -227,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -246,6 +246,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1125,13 +1126,13 @@
       </c>
       <c r="H2" s="4">
         <f>K2</f>
-        <v>50.75</v>
+        <v>55.67</v>
       </c>
       <c r="J2" s="2">
         <v>20</v>
       </c>
-      <c r="K2" s="4">
-        <v>50.75</v>
+      <c r="K2" s="16">
+        <v>55.67</v>
       </c>
       <c r="L2" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Bulk commit. Lots of work
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -1,19 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47265F0-F091-4EC3-A720-CE5A303792C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
     <sheet name="FeedMgmt" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -157,7 +169,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -227,19 +239,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -526,8 +536,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -539,7 +549,7 @@
     <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
@@ -571,7 +581,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -586,23 +596,20 @@
       </c>
       <c r="H2" s="1">
         <f>K2</f>
-        <v>9576</v>
-      </c>
-      <c r="J2" s="13">
-        <v>10025.4</v>
-      </c>
-      <c r="K2" s="14">
-        <v>9576</v>
+        <v>9275.6691729323302</v>
+      </c>
+      <c r="J2" s="11">
+        <v>9638</v>
+      </c>
+      <c r="K2" s="12">
+        <f>J2/(K23/J23)</f>
+        <v>9275.6691729323302</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
       </c>
-      <c r="O2">
-        <f>K2/J2</f>
-        <v>0.95517385839966484</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -617,23 +624,20 @@
       </c>
       <c r="H3" s="1">
         <f>K3</f>
-        <v>8960</v>
-      </c>
-      <c r="J3" s="13">
-        <v>9367.2000000000007</v>
-      </c>
-      <c r="K3" s="14">
-        <v>8960</v>
+        <v>8676.350364963504</v>
+      </c>
+      <c r="J3" s="11">
+        <v>9005</v>
+      </c>
+      <c r="K3" s="12">
+        <f>J3/(K24/J24)</f>
+        <v>8676.350364963504</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
-      <c r="O3">
-        <f>K3/J3</f>
-        <v>0.95652916559911172</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -648,20 +652,20 @@
       </c>
       <c r="H5" s="1">
         <f>K5</f>
-        <v>13.81875</v>
+        <v>13.715625000000001</v>
       </c>
       <c r="J5">
         <v>13.2</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="10">
         <f>12 / (K25 / (K23/12))</f>
-        <v>13.81875</v>
+        <v>13.715625000000001</v>
       </c>
       <c r="L5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -676,20 +680,20 @@
       </c>
       <c r="H6" s="1">
         <f>K6</f>
-        <v>13.486363636363636</v>
+        <v>13.388636363636362</v>
       </c>
       <c r="J6">
         <v>12.9</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="10">
         <f>12 / (K26 / (K24/12))</f>
-        <v>13.486363636363636</v>
+        <v>13.388636363636362</v>
       </c>
       <c r="L6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -704,19 +708,20 @@
       </c>
       <c r="H8" s="1">
         <f>K8</f>
-        <v>35.799999999999997</v>
+        <v>36.090225563909769</v>
       </c>
       <c r="J8">
         <v>37.1</v>
       </c>
-      <c r="K8" s="11">
-        <v>35.799999999999997</v>
+      <c r="K8" s="10">
+        <f>12/K23*100</f>
+        <v>36.090225563909769</v>
       </c>
       <c r="L8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -731,19 +736,20 @@
       </c>
       <c r="H9" s="1">
         <f>K9</f>
-        <v>34.799999999999997</v>
+        <v>35.036496350364963</v>
       </c>
       <c r="J9">
         <v>36.1</v>
       </c>
-      <c r="K9" s="11">
-        <v>34.799999999999997</v>
+      <c r="K9" s="10">
+        <f>12/K24*100</f>
+        <v>35.036496350364963</v>
       </c>
       <c r="L9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -766,16 +772,15 @@
       <c r="J11" s="4">
         <v>651.52821361702138</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="8">
         <f>J11</f>
         <v>651.52821361702138</v>
       </c>
       <c r="L11" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="6"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -786,9 +791,8 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="4"/>
-      <c r="M12" s="6"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>32</v>
       </c>
@@ -802,9 +806,8 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="4"/>
-      <c r="M13" s="6"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -822,19 +825,19 @@
       </c>
       <c r="H14" s="1">
         <f>K14</f>
-        <v>10.721</v>
+        <v>10.1</v>
       </c>
       <c r="J14" s="1">
         <v>6.6079520088655128</v>
       </c>
-      <c r="K14" s="12">
-        <v>10.721</v>
+      <c r="K14" s="10">
+        <v>10.1</v>
       </c>
       <c r="L14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -847,15 +850,15 @@
       <c r="G15" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="6">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
-        <v>0.95446267697244147</v>
+        <v>0.96110165503447054</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -879,13 +882,13 @@
       </c>
       <c r="H16" s="1">
         <f>K16</f>
-        <v>10.721</v>
+        <v>10.1</v>
       </c>
       <c r="J16" s="1">
         <v>6.4615074492035101</v>
       </c>
-      <c r="K16" s="12">
-        <v>10.721</v>
+      <c r="K16" s="10">
+        <v>10.1</v>
       </c>
       <c r="L16" t="s">
         <v>26</v>
@@ -910,16 +913,16 @@
       <c r="G17" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="6">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
-        <v>0.95446267697244147</v>
+        <v>0.96110165503447054</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="7" t="s">
         <v>39</v>
       </c>
       <c r="I19" t="s">
@@ -928,7 +931,7 @@
       <c r="J19">
         <v>0</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19" s="9">
         <v>0.25</v>
       </c>
       <c r="L19" t="s">
@@ -942,7 +945,7 @@
       <c r="J20">
         <v>0</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20" s="9">
         <v>0.25</v>
       </c>
       <c r="L20" t="s">
@@ -950,7 +953,7 @@
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="7" t="s">
         <v>38</v>
       </c>
       <c r="I21" t="s">
@@ -959,8 +962,8 @@
       <c r="J21">
         <v>0</v>
       </c>
-      <c r="K21" s="11">
-        <v>6</v>
+      <c r="K21" s="9">
+        <v>5</v>
       </c>
       <c r="L21" t="s">
         <v>27</v>
@@ -973,15 +976,15 @@
       <c r="J22">
         <v>0</v>
       </c>
-      <c r="K22" s="11">
-        <v>6</v>
+      <c r="K22" s="9">
+        <v>5</v>
       </c>
       <c r="L22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="7" t="s">
         <v>34</v>
       </c>
       <c r="I23" t="s">
@@ -990,9 +993,9 @@
       <c r="J23" s="1">
         <v>32</v>
       </c>
-      <c r="K23" s="12">
+      <c r="K23" s="10">
         <f>J23+K21*K19</f>
-        <v>33.5</v>
+        <v>33.25</v>
       </c>
       <c r="L23" t="s">
         <v>27</v>
@@ -1005,9 +1008,9 @@
       <c r="J24" s="1">
         <v>33</v>
       </c>
-      <c r="K24" s="12">
+      <c r="K24" s="10">
         <f>J24+K22*K20</f>
-        <v>34.5</v>
+        <v>34.25</v>
       </c>
       <c r="L24" t="s">
         <v>27</v>
@@ -1024,7 +1027,7 @@
         <f>(12/J5) * (J23/12)</f>
         <v>2.4242424242424243</v>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="13">
         <f>J25</f>
         <v>2.4242424242424243</v>
       </c>
@@ -1040,7 +1043,7 @@
         <f>(12/J6) * (J24/12)</f>
         <v>2.558139534883721</v>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="13">
         <f>J26</f>
         <v>2.558139534883721</v>
       </c>
@@ -1055,7 +1058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1098,7 +1101,7 @@
       <c r="J1" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1126,13 +1129,13 @@
       </c>
       <c r="H2" s="4">
         <f>K2</f>
-        <v>55.67</v>
+        <v>53</v>
       </c>
       <c r="J2" s="2">
         <v>20</v>
       </c>
-      <c r="K2" s="16">
-        <v>55.67</v>
+      <c r="K2" s="14">
+        <v>53</v>
       </c>
       <c r="L2" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Small fix not affecting scenario
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47265F0-F091-4EC3-A720-CE5A303792C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE46BD2-ADF1-4E3B-951F-07F470A84433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
@@ -1132,7 +1132,7 @@
         <v>53</v>
       </c>
       <c r="J2" s="2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="K2" s="14">
         <v>53</v>

</xml_diff>

<commit_message>
Fixed misstake in parameter name 'replacement_rate'
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE46BD2-ADF1-4E3B-951F-07F470A84433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C64D303-F47B-44B3-955D-FCE074784CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1965" yWindow="2115" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
@@ -85,9 +85,6 @@
     <t>orig.</t>
   </si>
   <si>
-    <t>recruitment_rate</t>
-  </si>
-  <si>
     <t>cattle</t>
   </si>
   <si>
@@ -164,6 +161,9 @@
   </si>
   <si>
     <t>frac.</t>
+  </si>
+  <si>
+    <t>replacement_rate</t>
   </si>
 </sst>
 </file>
@@ -557,7 +557,7 @@
         <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>8</v>
@@ -578,7 +578,7 @@
         <v>16</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -606,7 +606,7 @@
         <v>9275.6691729323302</v>
       </c>
       <c r="L2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -634,7 +634,7 @@
         <v>8676.350364963504</v>
       </c>
       <c r="L3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -662,7 +662,7 @@
         <v>13.715625000000001</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -690,7 +690,7 @@
         <v>13.388636363636362</v>
       </c>
       <c r="L6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -701,7 +701,7 @@
         <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="G8" t="s">
         <v>2</v>
@@ -718,7 +718,7 @@
         <v>36.090225563909769</v>
       </c>
       <c r="L8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -729,7 +729,7 @@
         <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s">
         <v>2</v>
@@ -746,7 +746,7 @@
         <v>35.036496350364963</v>
       </c>
       <c r="L9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -759,7 +759,7 @@
         <v>5</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>2</v>
@@ -777,7 +777,7 @@
         <v>651.52821361702138</v>
       </c>
       <c r="L11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -794,7 +794,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -834,7 +834,7 @@
         <v>10.1</v>
       </c>
       <c r="L14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -848,14 +848,14 @@
         <v>6</v>
       </c>
       <c r="G15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H15" s="6">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
         <v>0.96110165503447054</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -866,7 +866,7 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -891,7 +891,7 @@
         <v>10.1</v>
       </c>
       <c r="L16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -902,7 +902,7 @@
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -911,22 +911,22 @@
         <v>6</v>
       </c>
       <c r="G17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H17" s="6">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
         <v>0.96110165503447054</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H19" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -935,12 +935,12 @@
         <v>0.25</v>
       </c>
       <c r="L19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -949,15 +949,15 @@
         <v>0.25</v>
       </c>
       <c r="L20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H21" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -966,12 +966,12 @@
         <v>5</v>
       </c>
       <c r="L21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -980,15 +980,15 @@
         <v>5</v>
       </c>
       <c r="L22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H23" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I23" t="s">
         <v>34</v>
-      </c>
-      <c r="I23" t="s">
-        <v>35</v>
       </c>
       <c r="J23" s="1">
         <v>32</v>
@@ -998,12 +998,12 @@
         <v>33.25</v>
       </c>
       <c r="L23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J24" s="1">
         <v>33</v>
@@ -1013,15 +1013,15 @@
         <v>34.25</v>
       </c>
       <c r="L24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J25" s="1">
         <f>(12/J5) * (J23/12)</f>
@@ -1032,12 +1032,12 @@
         <v>2.4242424242424243</v>
       </c>
       <c r="L25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J26" s="1">
         <f>(12/J6) * (J24/12)</f>
@@ -1048,7 +1048,7 @@
         <v>2.558139534883721</v>
       </c>
       <c r="L26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1075,7 +1075,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>9</v>
@@ -1084,10 +1084,10 @@
         <v>8</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>0</v>
@@ -1102,12 +1102,12 @@
         <v>16</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1116,13 +1116,13 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
         <v>2</v>
@@ -1138,10 +1138,10 @@
         <v>53</v>
       </c>
       <c r="L2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed minor things in scenarios
</commit_message>
<xml_diff>
--- a/scenarios/CUL_COWS.xlsx
+++ b/scenarios/CUL_COWS.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C64D303-F47B-44B3-955D-FCE074784CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551B7B53-A231-4A86-8574-E32EA7DE6D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1965" yWindow="2115" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19305" yWindow="-2775" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="45">
   <si>
     <t>parameter</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>replacement_rate</t>
+  </si>
+  <si>
+    <t>&lt;-- Same %-unit increase as conventional</t>
   </si>
 </sst>
 </file>
@@ -173,7 +176,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,6 +221,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -239,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -257,6 +268,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -594,7 +606,7 @@
       <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="4">
         <f>K2</f>
         <v>9275.6691729323302</v>
       </c>
@@ -602,7 +614,7 @@
         <v>9638</v>
       </c>
       <c r="K2" s="12">
-        <f>J2/(K23/J23)</f>
+        <f>J2/(K25/J25)</f>
         <v>9275.6691729323302</v>
       </c>
       <c r="L2" t="s">
@@ -622,7 +634,7 @@
       <c r="G3" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="4">
         <f>K3</f>
         <v>8676.350364963504</v>
       </c>
@@ -630,7 +642,7 @@
         <v>9005</v>
       </c>
       <c r="K3" s="12">
-        <f>J3/(K24/J24)</f>
+        <f>J3/(K26/J26)</f>
         <v>8676.350364963504</v>
       </c>
       <c r="L3" t="s">
@@ -658,7 +670,7 @@
         <v>13.2</v>
       </c>
       <c r="K5" s="10">
-        <f>12 / (K25 / (K23/12))</f>
+        <f>12 / (K27 / (K25/12))</f>
         <v>13.715625000000001</v>
       </c>
       <c r="L5" t="s">
@@ -686,7 +698,7 @@
         <v>12.9</v>
       </c>
       <c r="K6" s="10">
-        <f>12 / (K26 / (K24/12))</f>
+        <f>12 / (K28 / (K26/12))</f>
         <v>13.388636363636362</v>
       </c>
       <c r="L6" t="s">
@@ -714,7 +726,7 @@
         <v>37.1</v>
       </c>
       <c r="K8" s="10">
-        <f>12/K23*100</f>
+        <f>12/K25*100</f>
         <v>36.090225563909769</v>
       </c>
       <c r="L8" t="s">
@@ -742,7 +754,7 @@
         <v>36.1</v>
       </c>
       <c r="K9" s="10">
-        <f>12/K24*100</f>
+        <f>12/K26*100</f>
         <v>35.036496350364963</v>
       </c>
       <c r="L9" t="s">
@@ -811,6 +823,9 @@
       <c r="A14" t="s">
         <v>4</v>
       </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
       <c r="D14" t="s">
         <v>5</v>
       </c>
@@ -841,6 +856,9 @@
       <c r="A15" t="s">
         <v>4</v>
       </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
       <c r="D15" t="s">
         <v>5</v>
       </c>
@@ -851,7 +869,7 @@
         <v>32</v>
       </c>
       <c r="H15" s="6">
-        <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
+        <f>(1 / (100 - J$18)) * (1 - K$18/100) * 100</f>
         <v>0.96110165503447054</v>
       </c>
       <c r="J15" s="1" t="s">
@@ -863,10 +881,7 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -882,16 +897,17 @@
       </c>
       <c r="H16" s="1">
         <f>K16</f>
-        <v>10.1</v>
+        <v>14.289458206396507</v>
       </c>
       <c r="J16" s="1">
-        <v>6.4615074492035101</v>
+        <v>10.797410215262019</v>
       </c>
       <c r="K16" s="10">
-        <v>10.1</v>
-      </c>
-      <c r="L16" t="s">
-        <v>25</v>
+        <f>J16+(K14-J14)</f>
+        <v>14.289458206396507</v>
+      </c>
+      <c r="L16" s="15" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -899,10 +915,7 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -915,46 +928,78 @@
       </c>
       <c r="H17" s="6">
         <f>(1 / (100 - J$16)) * (1 - K$16/100) * 100</f>
-        <v>0.96110165503447054</v>
+        <v>0.9608526165040564</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>40</v>
       </c>
     </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" t="s">
+        <v>2</v>
+      </c>
+      <c r="H18" s="1">
+        <f>K18</f>
+        <v>10.1</v>
+      </c>
+      <c r="J18" s="1">
+        <v>6.4615074492035101</v>
+      </c>
+      <c r="K18" s="10">
+        <v>10.1</v>
+      </c>
+      <c r="L18" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H19" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I19" t="s">
-        <v>34</v>
-      </c>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19" s="9">
-        <v>0.25</v>
-      </c>
-      <c r="L19" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="I20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20" s="9">
-        <v>0.25</v>
-      </c>
-      <c r="L20" t="s">
-        <v>42</v>
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>6</v>
+      </c>
+      <c r="G19" t="s">
+        <v>32</v>
+      </c>
+      <c r="H19" s="6">
+        <f>(1 / (100 - J$18)) * (1 - K$18/100) * 100</f>
+        <v>0.96110165503447054</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H21" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I21" t="s">
         <v>34</v>
@@ -963,10 +1008,10 @@
         <v>0</v>
       </c>
       <c r="K21" s="9">
-        <v>5</v>
+        <v>0.25</v>
       </c>
       <c r="L21" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -977,25 +1022,24 @@
         <v>0</v>
       </c>
       <c r="K22" s="9">
-        <v>5</v>
+        <v>0.25</v>
       </c>
       <c r="L22" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H23" s="7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I23" t="s">
         <v>34</v>
       </c>
-      <c r="J23" s="1">
-        <v>32</v>
-      </c>
-      <c r="K23" s="10">
-        <f>J23+K21*K19</f>
-        <v>33.25</v>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23" s="9">
+        <v>5</v>
       </c>
       <c r="L23" t="s">
         <v>26</v>
@@ -1005,34 +1049,32 @@
       <c r="I24" t="s">
         <v>35</v>
       </c>
-      <c r="J24" s="1">
-        <v>33</v>
-      </c>
-      <c r="K24" s="10">
-        <f>J24+K22*K20</f>
-        <v>34.25</v>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24" s="9">
+        <v>5</v>
       </c>
       <c r="L24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H25" t="s">
-        <v>36</v>
+      <c r="H25" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="I25" t="s">
         <v>34</v>
       </c>
       <c r="J25" s="1">
-        <f>(12/J5) * (J23/12)</f>
-        <v>2.4242424242424243</v>
-      </c>
-      <c r="K25" s="13">
-        <f>J25</f>
-        <v>2.4242424242424243</v>
+        <v>32</v>
+      </c>
+      <c r="K25" s="10">
+        <f>J25+K23*K21</f>
+        <v>33.25</v>
       </c>
       <c r="L25" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -1040,14 +1082,48 @@
         <v>35</v>
       </c>
       <c r="J26" s="1">
-        <f>(12/J6) * (J24/12)</f>
+        <v>33</v>
+      </c>
+      <c r="K26" s="10">
+        <f>J26+K24*K22</f>
+        <v>34.25</v>
+      </c>
+      <c r="L26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" t="s">
+        <v>34</v>
+      </c>
+      <c r="J27" s="1">
+        <f>(12/J5) * (J25/12)</f>
+        <v>2.4242424242424243</v>
+      </c>
+      <c r="K27" s="13">
+        <f>J27</f>
+        <v>2.4242424242424243</v>
+      </c>
+      <c r="L27" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I28" t="s">
+        <v>35</v>
+      </c>
+      <c r="J28" s="1">
+        <f>(12/J6) * (J26/12)</f>
         <v>2.558139534883721</v>
       </c>
-      <c r="K26" s="13">
-        <f>J26</f>
+      <c r="K28" s="13">
+        <f>J28</f>
         <v>2.558139534883721</v>
       </c>
-      <c r="L26" t="s">
+      <c r="L28" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>